<commit_message>
Review: cuatro correcciones de CodeRabbit en la calculadora y la planilla
- Planilla: una fila con "Facturable" vacío sumaba al importe pero no a las
  horas facturables del resumen. Las dos columnas usan ahora el mismo
  criterio (todo lo que no es "No" cuenta como facturable).
- Calculadora de horas: las horas en decimal se muestran siempre con coma,
  como el resto de la página; con USD el locale en-US las mostraba con
  punto. La FAQ sobre sumar horas y minutos se contradecía (15 horas y 55
  minutos es 15:55): queda el ejemplo con y sin acarreo.
- Post de control de horas: los parciales por día y el promedio de 4:45
  son horas trabajadas, no facturables (las facturables promedian 4:33).

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BpQVenqBUqXFbBbk4NGLPi
</commit_message>
<xml_diff>
--- a/public/plantillas/control-de-horas-trabajadas.xlsx
+++ b/public/plantillas/control-de-horas-trabajadas.xlsx
@@ -10850,7 +10850,7 @@
         <v/>
       </c>
       <c r="C5" s="5">
-        <f>IF(A5="","",SUMIFS(Horas!$G:$G,Horas!$B:$B,A5,Horas!$I:$I,"Sí"))</f>
+        <f>IF(A5="","",SUMIFS(Horas!$G:$G,Horas!$B:$B,A5,Horas!$I:$I,"&lt;&gt;No"))</f>
         <v/>
       </c>
       <c r="D5" s="11">
@@ -10868,7 +10868,7 @@
         <v/>
       </c>
       <c r="C6" s="5">
-        <f>IF(A6="","",SUMIFS(Horas!$G:$G,Horas!$B:$B,A6,Horas!$I:$I,"Sí"))</f>
+        <f>IF(A6="","",SUMIFS(Horas!$G:$G,Horas!$B:$B,A6,Horas!$I:$I,"&lt;&gt;No"))</f>
         <v/>
       </c>
       <c r="D6" s="11">
@@ -10886,7 +10886,7 @@
         <v/>
       </c>
       <c r="C7" s="5">
-        <f>IF(A7="","",SUMIFS(Horas!$G:$G,Horas!$B:$B,A7,Horas!$I:$I,"Sí"))</f>
+        <f>IF(A7="","",SUMIFS(Horas!$G:$G,Horas!$B:$B,A7,Horas!$I:$I,"&lt;&gt;No"))</f>
         <v/>
       </c>
       <c r="D7" s="11">
@@ -10904,7 +10904,7 @@
         <v/>
       </c>
       <c r="C8" s="5">
-        <f>IF(A8="","",SUMIFS(Horas!$G:$G,Horas!$B:$B,A8,Horas!$I:$I,"Sí"))</f>
+        <f>IF(A8="","",SUMIFS(Horas!$G:$G,Horas!$B:$B,A8,Horas!$I:$I,"&lt;&gt;No"))</f>
         <v/>
       </c>
       <c r="D8" s="11">
@@ -10922,7 +10922,7 @@
         <v/>
       </c>
       <c r="C9" s="5">
-        <f>IF(A9="","",SUMIFS(Horas!$G:$G,Horas!$B:$B,A9,Horas!$I:$I,"Sí"))</f>
+        <f>IF(A9="","",SUMIFS(Horas!$G:$G,Horas!$B:$B,A9,Horas!$I:$I,"&lt;&gt;No"))</f>
         <v/>
       </c>
       <c r="D9" s="11">
@@ -10940,7 +10940,7 @@
         <v/>
       </c>
       <c r="C10" s="5">
-        <f>IF(A10="","",SUMIFS(Horas!$G:$G,Horas!$B:$B,A10,Horas!$I:$I,"Sí"))</f>
+        <f>IF(A10="","",SUMIFS(Horas!$G:$G,Horas!$B:$B,A10,Horas!$I:$I,"&lt;&gt;No"))</f>
         <v/>
       </c>
       <c r="D10" s="11">
@@ -10958,7 +10958,7 @@
         <v/>
       </c>
       <c r="C11" s="5">
-        <f>IF(A11="","",SUMIFS(Horas!$G:$G,Horas!$B:$B,A11,Horas!$I:$I,"Sí"))</f>
+        <f>IF(A11="","",SUMIFS(Horas!$G:$G,Horas!$B:$B,A11,Horas!$I:$I,"&lt;&gt;No"))</f>
         <v/>
       </c>
       <c r="D11" s="11">
@@ -10976,7 +10976,7 @@
         <v/>
       </c>
       <c r="C12" s="5">
-        <f>IF(A12="","",SUMIFS(Horas!$G:$G,Horas!$B:$B,A12,Horas!$I:$I,"Sí"))</f>
+        <f>IF(A12="","",SUMIFS(Horas!$G:$G,Horas!$B:$B,A12,Horas!$I:$I,"&lt;&gt;No"))</f>
         <v/>
       </c>
       <c r="D12" s="11">
@@ -10994,7 +10994,7 @@
         <v/>
       </c>
       <c r="C13" s="5">
-        <f>IF(A13="","",SUMIFS(Horas!$G:$G,Horas!$B:$B,A13,Horas!$I:$I,"Sí"))</f>
+        <f>IF(A13="","",SUMIFS(Horas!$G:$G,Horas!$B:$B,A13,Horas!$I:$I,"&lt;&gt;No"))</f>
         <v/>
       </c>
       <c r="D13" s="11">
@@ -11012,7 +11012,7 @@
         <v/>
       </c>
       <c r="C14" s="5">
-        <f>IF(A14="","",SUMIFS(Horas!$G:$G,Horas!$B:$B,A14,Horas!$I:$I,"Sí"))</f>
+        <f>IF(A14="","",SUMIFS(Horas!$G:$G,Horas!$B:$B,A14,Horas!$I:$I,"&lt;&gt;No"))</f>
         <v/>
       </c>
       <c r="D14" s="11">
@@ -11030,7 +11030,7 @@
         <v/>
       </c>
       <c r="C15" s="5">
-        <f>IF(A15="","",SUMIFS(Horas!$G:$G,Horas!$B:$B,A15,Horas!$I:$I,"Sí"))</f>
+        <f>IF(A15="","",SUMIFS(Horas!$G:$G,Horas!$B:$B,A15,Horas!$I:$I,"&lt;&gt;No"))</f>
         <v/>
       </c>
       <c r="D15" s="11">
@@ -11048,7 +11048,7 @@
         <v/>
       </c>
       <c r="C16" s="5">
-        <f>IF(A16="","",SUMIFS(Horas!$G:$G,Horas!$B:$B,A16,Horas!$I:$I,"Sí"))</f>
+        <f>IF(A16="","",SUMIFS(Horas!$G:$G,Horas!$B:$B,A16,Horas!$I:$I,"&lt;&gt;No"))</f>
         <v/>
       </c>
       <c r="D16" s="11">
@@ -11066,7 +11066,7 @@
         <v/>
       </c>
       <c r="C17" s="5">
-        <f>IF(A17="","",SUMIFS(Horas!$G:$G,Horas!$B:$B,A17,Horas!$I:$I,"Sí"))</f>
+        <f>IF(A17="","",SUMIFS(Horas!$G:$G,Horas!$B:$B,A17,Horas!$I:$I,"&lt;&gt;No"))</f>
         <v/>
       </c>
       <c r="D17" s="11">
@@ -11084,7 +11084,7 @@
         <v/>
       </c>
       <c r="C18" s="5">
-        <f>IF(A18="","",SUMIFS(Horas!$G:$G,Horas!$B:$B,A18,Horas!$I:$I,"Sí"))</f>
+        <f>IF(A18="","",SUMIFS(Horas!$G:$G,Horas!$B:$B,A18,Horas!$I:$I,"&lt;&gt;No"))</f>
         <v/>
       </c>
       <c r="D18" s="11">
@@ -11102,7 +11102,7 @@
         <v/>
       </c>
       <c r="C19" s="5">
-        <f>IF(A19="","",SUMIFS(Horas!$G:$G,Horas!$B:$B,A19,Horas!$I:$I,"Sí"))</f>
+        <f>IF(A19="","",SUMIFS(Horas!$G:$G,Horas!$B:$B,A19,Horas!$I:$I,"&lt;&gt;No"))</f>
         <v/>
       </c>
       <c r="D19" s="11">
@@ -11120,7 +11120,7 @@
         <v/>
       </c>
       <c r="C20" s="5">
-        <f>IF(A20="","",SUMIFS(Horas!$G:$G,Horas!$B:$B,A20,Horas!$I:$I,"Sí"))</f>
+        <f>IF(A20="","",SUMIFS(Horas!$G:$G,Horas!$B:$B,A20,Horas!$I:$I,"&lt;&gt;No"))</f>
         <v/>
       </c>
       <c r="D20" s="11">
@@ -11138,7 +11138,7 @@
         <v/>
       </c>
       <c r="C21" s="5">
-        <f>IF(A21="","",SUMIFS(Horas!$G:$G,Horas!$B:$B,A21,Horas!$I:$I,"Sí"))</f>
+        <f>IF(A21="","",SUMIFS(Horas!$G:$G,Horas!$B:$B,A21,Horas!$I:$I,"&lt;&gt;No"))</f>
         <v/>
       </c>
       <c r="D21" s="11">
@@ -11156,7 +11156,7 @@
         <v/>
       </c>
       <c r="C22" s="5">
-        <f>IF(A22="","",SUMIFS(Horas!$G:$G,Horas!$B:$B,A22,Horas!$I:$I,"Sí"))</f>
+        <f>IF(A22="","",SUMIFS(Horas!$G:$G,Horas!$B:$B,A22,Horas!$I:$I,"&lt;&gt;No"))</f>
         <v/>
       </c>
       <c r="D22" s="11">
@@ -11174,7 +11174,7 @@
         <v/>
       </c>
       <c r="C23" s="5">
-        <f>IF(A23="","",SUMIFS(Horas!$G:$G,Horas!$B:$B,A23,Horas!$I:$I,"Sí"))</f>
+        <f>IF(A23="","",SUMIFS(Horas!$G:$G,Horas!$B:$B,A23,Horas!$I:$I,"&lt;&gt;No"))</f>
         <v/>
       </c>
       <c r="D23" s="11">
@@ -11192,7 +11192,7 @@
         <v/>
       </c>
       <c r="C24" s="5">
-        <f>IF(A24="","",SUMIFS(Horas!$G:$G,Horas!$B:$B,A24,Horas!$I:$I,"Sí"))</f>
+        <f>IF(A24="","",SUMIFS(Horas!$G:$G,Horas!$B:$B,A24,Horas!$I:$I,"&lt;&gt;No"))</f>
         <v/>
       </c>
       <c r="D24" s="11">
@@ -11210,7 +11210,7 @@
         <v/>
       </c>
       <c r="C25" s="5">
-        <f>IF(A25="","",SUMIFS(Horas!$G:$G,Horas!$B:$B,A25,Horas!$I:$I,"Sí"))</f>
+        <f>IF(A25="","",SUMIFS(Horas!$G:$G,Horas!$B:$B,A25,Horas!$I:$I,"&lt;&gt;No"))</f>
         <v/>
       </c>
       <c r="D25" s="11">
@@ -11228,7 +11228,7 @@
         <v/>
       </c>
       <c r="C26" s="5">
-        <f>IF(A26="","",SUMIFS(Horas!$G:$G,Horas!$B:$B,A26,Horas!$I:$I,"Sí"))</f>
+        <f>IF(A26="","",SUMIFS(Horas!$G:$G,Horas!$B:$B,A26,Horas!$I:$I,"&lt;&gt;No"))</f>
         <v/>
       </c>
       <c r="D26" s="11">
@@ -11246,7 +11246,7 @@
         <v/>
       </c>
       <c r="C27" s="5">
-        <f>IF(A27="","",SUMIFS(Horas!$G:$G,Horas!$B:$B,A27,Horas!$I:$I,"Sí"))</f>
+        <f>IF(A27="","",SUMIFS(Horas!$G:$G,Horas!$B:$B,A27,Horas!$I:$I,"&lt;&gt;No"))</f>
         <v/>
       </c>
       <c r="D27" s="11">
@@ -11264,7 +11264,7 @@
         <v/>
       </c>
       <c r="C28" s="5">
-        <f>IF(A28="","",SUMIFS(Horas!$G:$G,Horas!$B:$B,A28,Horas!$I:$I,"Sí"))</f>
+        <f>IF(A28="","",SUMIFS(Horas!$G:$G,Horas!$B:$B,A28,Horas!$I:$I,"&lt;&gt;No"))</f>
         <v/>
       </c>
       <c r="D28" s="11">
@@ -11282,7 +11282,7 @@
         <v/>
       </c>
       <c r="C29" s="5">
-        <f>IF(A29="","",SUMIFS(Horas!$G:$G,Horas!$B:$B,A29,Horas!$I:$I,"Sí"))</f>
+        <f>IF(A29="","",SUMIFS(Horas!$G:$G,Horas!$B:$B,A29,Horas!$I:$I,"&lt;&gt;No"))</f>
         <v/>
       </c>
       <c r="D29" s="11">
@@ -11300,7 +11300,7 @@
         <v/>
       </c>
       <c r="C30" s="5">
-        <f>IF(A30="","",SUMIFS(Horas!$G:$G,Horas!$B:$B,A30,Horas!$I:$I,"Sí"))</f>
+        <f>IF(A30="","",SUMIFS(Horas!$G:$G,Horas!$B:$B,A30,Horas!$I:$I,"&lt;&gt;No"))</f>
         <v/>
       </c>
       <c r="D30" s="11">
@@ -11318,7 +11318,7 @@
         <v/>
       </c>
       <c r="C31" s="5">
-        <f>IF(A31="","",SUMIFS(Horas!$G:$G,Horas!$B:$B,A31,Horas!$I:$I,"Sí"))</f>
+        <f>IF(A31="","",SUMIFS(Horas!$G:$G,Horas!$B:$B,A31,Horas!$I:$I,"&lt;&gt;No"))</f>
         <v/>
       </c>
       <c r="D31" s="11">
@@ -11336,7 +11336,7 @@
         <v/>
       </c>
       <c r="C32" s="5">
-        <f>IF(A32="","",SUMIFS(Horas!$G:$G,Horas!$B:$B,A32,Horas!$I:$I,"Sí"))</f>
+        <f>IF(A32="","",SUMIFS(Horas!$G:$G,Horas!$B:$B,A32,Horas!$I:$I,"&lt;&gt;No"))</f>
         <v/>
       </c>
       <c r="D32" s="11">
@@ -11354,7 +11354,7 @@
         <v/>
       </c>
       <c r="C33" s="5">
-        <f>IF(A33="","",SUMIFS(Horas!$G:$G,Horas!$B:$B,A33,Horas!$I:$I,"Sí"))</f>
+        <f>IF(A33="","",SUMIFS(Horas!$G:$G,Horas!$B:$B,A33,Horas!$I:$I,"&lt;&gt;No"))</f>
         <v/>
       </c>
       <c r="D33" s="11">
@@ -11372,7 +11372,7 @@
         <v/>
       </c>
       <c r="C34" s="5">
-        <f>IF(A34="","",SUMIFS(Horas!$G:$G,Horas!$B:$B,A34,Horas!$I:$I,"Sí"))</f>
+        <f>IF(A34="","",SUMIFS(Horas!$G:$G,Horas!$B:$B,A34,Horas!$I:$I,"&lt;&gt;No"))</f>
         <v/>
       </c>
       <c r="D34" s="11">
@@ -11451,7 +11451,7 @@
         </is>
       </c>
       <c r="B42" s="5">
-        <f>SUMIFS(Horas!$G:$G,Horas!$A:$A,"&gt;="&amp;B39,Horas!$A:$A,"&lt;="&amp;B40,Horas!$I:$I,"Sí")</f>
+        <f>SUMIFS(Horas!$G:$G,Horas!$A:$A,"&gt;="&amp;B39,Horas!$A:$A,"&lt;="&amp;B40,Horas!$I:$I,"&lt;&gt;No")</f>
         <v/>
       </c>
     </row>
@@ -11760,7 +11760,7 @@
     <row r="6">
       <c r="A6" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">   El descanso va en formato de hora (0:45 son 45 minutos). Facturable: Sí o No.</t>
+          <t xml:space="preserve">   El descanso va en formato de hora (0:45 son 45 minutos). Facturable: Sí o No (vacío cuenta como Sí).</t>
         </is>
       </c>
     </row>

</xml_diff>